<commit_message>
Fixed inconsistency in MTT18 LAB1 (now fully)
</commit_message>
<xml_diff>
--- a/other-data/inclusion_sets.xlsx
+++ b/other-data/inclusion_sets.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olavobohreramaral/Dropbox/bri-analysis-pp-main/other-data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olavobohreramaral/Dropbox/bri-analysis-pp-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCC7A15-7516-F84B-92C3-1762C4ABB5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC8C075-9ED6-CB40-92B7-53C06B21DD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2353" uniqueCount="221">
   <si>
     <t>EXP</t>
   </si>
@@ -6146,10 +6146,16 @@
       <c r="F65" t="s">
         <v>103</v>
       </c>
+      <c r="H65" t="s">
+        <v>103</v>
+      </c>
       <c r="I65" t="s">
         <v>103</v>
       </c>
       <c r="J65" t="s">
+        <v>103</v>
+      </c>
+      <c r="K65" t="s">
         <v>103</v>
       </c>
       <c r="L65" t="s">

</xml_diff>